<commit_message>
AR Excel: limit paid sheet to docs still open in Autoline, add CR match comments
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011H6KRJ6RQdimu91ogpyiHm
</commit_message>
<xml_diff>
--- a/AR_All_2026-10-23.xlsx
+++ b/AR_All_2026-10-23.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'AR Open'!$A$1:$M$373</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Paid - CR match'!$A$3:$L$64</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Paid - CR match'!$A$3:$L$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2956" uniqueCount="1096">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2945" uniqueCount="1062">
   <si>
     <t xml:space="preserve">AR summary – Quick Lane (Co 26 basis, USD)</t>
   </si>
@@ -2821,7 +2821,7 @@
     <t xml:space="preserve">VLS-PO05380</t>
   </si>
   <si>
-    <t xml:space="preserve">Documents marked paid in Supabase but still on the Autoline ledger. Fill column K with the CR number from Suphutta (Kitty)'s email, then mark L = Yes.</t>
+    <t xml:space="preserve">Paid per Supabase but still shown as open in Autoline (checked 23/10 against pasted ledgers). Docs not on the ledger are not listed. Kitty's CR emails are not readable by Claude: only 6138417 is matched.</t>
   </si>
   <si>
     <t xml:space="preserve">Status</t>
@@ -2833,10 +2833,10 @@
     <t xml:space="preserve">Payment evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">CR no. (Kitty email)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matched?</t>
+    <t xml:space="preserve">CR match (Suphutta/Kitty)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment</t>
   </si>
   <si>
     <t xml:space="preserve">6131439</t>
@@ -2851,6 +2851,12 @@
     <t xml:space="preserve">LDB-LAK LAK 1945405 [Deposit to bank On 8 2026.xlsx / 12-14]</t>
   </si>
   <si>
+    <t xml:space="preserve">Check amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR file LDB 12/08/2026 LAK 1,945,405 (~$86.27) is not $76.95: check if deposit covers other docs.</t>
+  </si>
+  <si>
     <t xml:space="preserve">6130649</t>
   </si>
   <si>
@@ -2863,6 +2869,12 @@
     <t xml:space="preserve">JDB-LAK LAK 3790000 [Deposit to bank On 2-2- 2026.xlsx / Sheet7]</t>
   </si>
   <si>
+    <t xml:space="preserve">Check CR no.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR file JDB 02/02/2026 LAK 3,790,000. Amount OK. No Kitty CR email number in system.</t>
+  </si>
+  <si>
     <t xml:space="preserve">6133365</t>
   </si>
   <si>
@@ -2875,6 +2887,12 @@
     <t xml:space="preserve">JDB-LAK LAK 704000 [Deposit to bank On 2-2- 2026.xlsx / Sheet7]</t>
   </si>
   <si>
+    <t xml:space="preserve">Check date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR file JDB 02/02/2026 LAK 704,000. Amount OK but invoice date 11/05/2026 is after deposit 02/02/2026: verify.</t>
+  </si>
+  <si>
     <t xml:space="preserve">6138417</t>
   </si>
   <si>
@@ -2884,151 +2902,31 @@
     <t xml:space="preserve">TT BCEL-LAK 1,934,790 (= USD 85.80 @22,550) deposit 09/10/26</t>
   </si>
   <si>
-    <t xml:space="preserve">6139259</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27656</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BORDALAOS</t>
+    <t xml:space="preserve">Matched</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATCHED Kitty CR email 22/10 (mail 590). TT BCEL 1,934,790 LAK = $85.80 @22,550. Still open in Autoline: Finance post receipt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6132877</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25764</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PO#4500542886</t>
   </si>
   <si>
     <t xml:space="preserve">paid (seen)</t>
   </si>
   <si>
-    <t xml:space="preserve">àºªàº»à»àºà»àº¡àº§15-10-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139309</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27557</t>
-  </si>
-  <si>
-    <t xml:space="preserve">àºªàº»à»àºà»àº¡àº§17-10-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139310</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27681</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VANHXAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139311</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27680</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KHAEK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139312</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27679</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TUNG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139314</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27667</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OLAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27620</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OLOTH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139318</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27637</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAPHANTHONG VILLAGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139319</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27611</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done Nakkhoum Villag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139320</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27686</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27689</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139336</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27695</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KHAMHOUNG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139338</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27699</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6138935</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">àºà»àº²àºà»àº¥à»àº§àºªàº»à»àºà»àº¡àº§21-10-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6137282</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THONGDOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">àºà»àº²àºà»àº¥à»àº§àºªàº»à»àºà»àº¡àº§20-10-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6132877</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25764</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PO#4500542886</t>
-  </si>
-  <si>
     <t xml:space="preserve">àºà»àº²àºà»àº¥à»àº§</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Need CR no.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid per AR comment 21/10 (Phubia 42-inv batch, $23,766.86, ql_kb #2434). No CR number in system: need Kitty CR email. Still open in Autoline: Finance post receipts.</t>
   </si>
   <si>
     <t xml:space="preserve">6133353</t>
@@ -3883,11 +3781,11 @@
         <v>27495.76</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A5)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A5)</f>
         <v>1</v>
       </c>
       <c r="H5" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A5)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A5)</f>
         <v>76.95</v>
       </c>
     </row>
@@ -3915,11 +3813,11 @@
         <v>0</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A6)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A6)</f>
         <v>0</v>
       </c>
       <c r="H6" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A6)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A6)</f>
         <v>0</v>
       </c>
     </row>
@@ -3947,11 +3845,11 @@
         <v>-118</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A7)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A7)</f>
         <v>42</v>
       </c>
       <c r="H7" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A7)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A7)</f>
         <v>23766.86</v>
       </c>
     </row>
@@ -3977,11 +3875,11 @@
         <v>0</v>
       </c>
       <c r="G8" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A8)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A8)</f>
         <v>0</v>
       </c>
       <c r="H8" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A8)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A8)</f>
         <v>0</v>
       </c>
     </row>
@@ -4007,11 +3905,11 @@
         <v>0</v>
       </c>
       <c r="G9" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A9)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A9)</f>
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A9)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A9)</f>
         <v>0</v>
       </c>
     </row>
@@ -4039,11 +3937,11 @@
         <v>1235.25</v>
       </c>
       <c r="G10" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A10)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A10)</f>
         <v>3</v>
       </c>
       <c r="H10" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A10)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A10)</f>
         <v>288.7</v>
       </c>
     </row>
@@ -4071,11 +3969,11 @@
         <v>-67.41</v>
       </c>
       <c r="G11" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A11)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A11)</f>
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A11)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A11)</f>
         <v>0</v>
       </c>
     </row>
@@ -4101,12 +3999,12 @@
         <v>0</v>
       </c>
       <c r="G12" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A12)</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A12)</f>
+        <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A12)</f>
-        <v>333.3</v>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A12)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4133,11 +4031,11 @@
         <v>0</v>
       </c>
       <c r="G13" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A13)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A13)</f>
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A13)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A13)</f>
         <v>0</v>
       </c>
     </row>
@@ -4165,12 +4063,12 @@
         <v>-78.09</v>
       </c>
       <c r="G14" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A14)</f>
-        <v>13</v>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A14)</f>
+        <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A14)</f>
-        <v>288.57</v>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A14)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4195,11 +4093,11 @@
         <v>1133.08</v>
       </c>
       <c r="G15" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A15)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A15)</f>
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A15)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A15)</f>
         <v>0</v>
       </c>
     </row>
@@ -4227,11 +4125,11 @@
         <v>0</v>
       </c>
       <c r="G16" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A16)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A16)</f>
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A16)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A16)</f>
         <v>0</v>
       </c>
     </row>
@@ -4259,11 +4157,11 @@
         <v>0</v>
       </c>
       <c r="G17" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A17)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A17)</f>
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A17)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A17)</f>
         <v>0</v>
       </c>
     </row>
@@ -4291,11 +4189,11 @@
         <v>-2060.81</v>
       </c>
       <c r="G18" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A18)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A18)</f>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A18)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A18)</f>
         <v>0</v>
       </c>
     </row>
@@ -4321,11 +4219,11 @@
         <v>0</v>
       </c>
       <c r="G19" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A19)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A19)</f>
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A19)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A19)</f>
         <v>0</v>
       </c>
     </row>
@@ -4351,11 +4249,11 @@
         <v>0</v>
       </c>
       <c r="G20" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A20)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A20)</f>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A20)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A20)</f>
         <v>0</v>
       </c>
     </row>
@@ -4381,11 +4279,11 @@
         <v>0</v>
       </c>
       <c r="G21" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A21)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A21)</f>
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A21)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A21)</f>
         <v>0</v>
       </c>
     </row>
@@ -4411,11 +4309,11 @@
         <v>61.6</v>
       </c>
       <c r="G22" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A22)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A22)</f>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A22)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A22)</f>
         <v>0</v>
       </c>
     </row>
@@ -4441,11 +4339,11 @@
         <v>0</v>
       </c>
       <c r="G23" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A23)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A23)</f>
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A23)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A23)</f>
         <v>0</v>
       </c>
     </row>
@@ -4471,11 +4369,11 @@
         <v>0</v>
       </c>
       <c r="G24" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A24)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A24)</f>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A24)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A24)</f>
         <v>0</v>
       </c>
     </row>
@@ -4501,11 +4399,11 @@
         <v>0</v>
       </c>
       <c r="G25" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A25)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A25)</f>
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A25)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A25)</f>
         <v>0</v>
       </c>
     </row>
@@ -4531,11 +4429,11 @@
         <v>0</v>
       </c>
       <c r="G26" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A26)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A26)</f>
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A26)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A26)</f>
         <v>0</v>
       </c>
     </row>
@@ -4561,12 +4459,12 @@
         <v>0</v>
       </c>
       <c r="G27" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A27)</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A27)</f>
+        <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A27)</f>
-        <v>75.06</v>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A27)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4591,11 +4489,11 @@
         <v>-4.65</v>
       </c>
       <c r="G28" s="5" t="n">
-        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$64,A28)</f>
+        <f aca="false">COUNTIFS('Paid - CR match'!$A$4:$A$49,A28)</f>
         <v>0</v>
       </c>
       <c r="H28" s="6" t="n">
-        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$64,'Paid - CR match'!$A$4:$A$64,A28)</f>
+        <f aca="false">SUMIFS('Paid - CR match'!$G$4:$G$49,'Paid - CR match'!$A$4:$A$49,A28)</f>
         <v>0</v>
       </c>
     </row>
@@ -4622,11 +4520,11 @@
       </c>
       <c r="G29" s="7" t="n">
         <f aca="false">SUM(G5:G28)</f>
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="H29" s="8" t="n">
         <f aca="false">SUM(H5:H28)</f>
-        <v>24829.44</v>
+        <v>24132.51</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20433,7 +20331,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -20444,9 +20342,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20454,7 +20352,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -20523,8 +20421,12 @@
       <c r="J4" s="5" t="s">
         <v>940</v>
       </c>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
+      <c r="K4" s="11" t="s">
+        <v>941</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>942</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -20534,13 +20436,13 @@
         <v>19</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>46007</v>
@@ -20555,10 +20457,14 @@
         <v>46063</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>944</v>
-      </c>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
+        <v>946</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>947</v>
+      </c>
+      <c r="L5" s="11" t="s">
+        <v>948</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -20568,13 +20474,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>46153</v>
@@ -20589,10 +20495,14 @@
         <v>46063</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>948</v>
-      </c>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
+        <v>952</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>953</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>954</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -20602,10 +20512,10 @@
         <v>19</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>643</v>
@@ -20623,486 +20533,554 @@
         <v>46304</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>951</v>
-      </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
+        <v>957</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>958</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>959</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>952</v>
+        <v>960</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>953</v>
+        <v>961</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>954</v>
+        <v>962</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>46310</v>
+        <v>46139</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>22</v>
+        <v>216.88</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="5" t="s">
-        <v>956</v>
-      </c>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>957</v>
+        <v>967</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>958</v>
+        <v>968</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>697</v>
+        <v>969</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>46312</v>
+        <v>46153</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>44</v>
+        <v>863</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>960</v>
+        <v>970</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>961</v>
+        <v>971</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>962</v>
+        <v>972</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>46312</v>
+        <v>46153</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4.43</v>
+        <v>340</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>973</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>974</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>972</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>46153</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>340</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>963</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>964</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>965</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>46312</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>69.3</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>955</v>
       </c>
       <c r="I11" s="10"/>
       <c r="J11" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>966</v>
+        <v>975</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>967</v>
+        <v>976</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>968</v>
+        <v>977</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>46312</v>
+        <v>46160</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>53.35</v>
+        <v>2469.91</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I12" s="10"/>
       <c r="J12" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>969</v>
+        <v>978</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>970</v>
+        <v>979</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>971</v>
+        <v>980</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>46312</v>
+        <v>46160</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>6.6</v>
+        <v>300</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I13" s="10"/>
       <c r="J13" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>972</v>
+        <v>981</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>973</v>
+        <v>982</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>46312</v>
+        <v>46160</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>16.5</v>
+        <v>138.4</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I14" s="10"/>
       <c r="J14" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>975</v>
+        <v>983</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>976</v>
+        <v>984</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>977</v>
       </c>
       <c r="F15" s="10" t="n">
-        <v>46312</v>
+        <v>46160</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>4.43</v>
+        <v>211.81</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I15" s="10"/>
       <c r="J15" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>978</v>
+        <v>985</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>979</v>
+        <v>986</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>46312</v>
+        <v>46160</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>4.4</v>
+        <v>1129.76</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>977</v>
+        <v>980</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>46312</v>
+        <v>46162</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>4.4</v>
+        <v>139.78</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>977</v>
+        <v>980</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>46312</v>
+        <v>46170</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>4.43</v>
+        <v>485.13</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I18" s="10"/>
       <c r="J18" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>987</v>
+        <v>808</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>46314</v>
+        <v>46198</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>50.33</v>
+        <v>1068.45</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I19" s="10"/>
       <c r="J19" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>980</v>
+        <v>995</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>46314</v>
+        <v>46198</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>4.4</v>
+        <v>316.46</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I20" s="10"/>
       <c r="J20" s="5" t="s">
-        <v>959</v>
-      </c>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L20" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="5"/>
+        <v>14</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="C21" s="5" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>748</v>
+        <v>995</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>46301</v>
+        <v>46198</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>333.3</v>
+        <v>309.58</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" s="5" t="s">
-        <v>992</v>
-      </c>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="5"/>
+        <v>14</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="C22" s="5" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>995</v>
+        <v>808</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>46256</v>
+        <v>46198</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>75.06</v>
+        <v>438.8</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I22" s="10"/>
       <c r="J22" s="5" t="s">
-        <v>996</v>
-      </c>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L22" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
@@ -21112,29 +21090,33 @@
         <v>15</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>997</v>
+        <v>1000</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>998</v>
+        <v>1001</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>999</v>
+        <v>1002</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>46139</v>
+        <v>46198</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>216.88</v>
+        <v>350.4</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I23" s="10"/>
       <c r="J23" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
@@ -21144,29 +21126,33 @@
         <v>15</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>46153</v>
+        <v>46198</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>863</v>
+        <v>149.16</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I24" s="10"/>
       <c r="J24" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K24" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L24" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
@@ -21176,29 +21162,33 @@
         <v>15</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>1006</v>
+        <v>995</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>46153</v>
+        <v>46198</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>340</v>
+        <v>309.58</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I25" s="10"/>
       <c r="J25" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
@@ -21208,29 +21198,33 @@
         <v>15</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>1006</v>
+        <v>808</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>46153</v>
+        <v>46198</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>340</v>
+        <v>837.52</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L26" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
@@ -21240,29 +21234,33 @@
         <v>15</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>1011</v>
+        <v>808</v>
       </c>
       <c r="F27" s="10" t="n">
-        <v>46160</v>
+        <v>46198</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>2469.91</v>
+        <v>610.85</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I27" s="10"/>
       <c r="J27" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L27" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
@@ -21281,20 +21279,24 @@
         <v>1014</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>46160</v>
+        <v>46198</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>300</v>
+        <v>1617.71</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I28" s="10"/>
       <c r="J28" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
@@ -21310,23 +21312,27 @@
         <v>1016</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>1014</v>
+        <v>995</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>46160</v>
+        <v>46198</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>138.4</v>
+        <v>300</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L29" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
@@ -21342,23 +21348,27 @@
         <v>1018</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>1011</v>
+        <v>995</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>46160</v>
+        <v>46198</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>211.81</v>
+        <v>527.8</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I30" s="10"/>
       <c r="J30" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
@@ -21374,23 +21384,27 @@
         <v>1020</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>1011</v>
+        <v>995</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>46160</v>
+        <v>46198</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>1129.76</v>
+        <v>494.11</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I31" s="10"/>
       <c r="J31" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
@@ -21406,23 +21420,27 @@
         <v>1022</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>1014</v>
+        <v>995</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>46162</v>
+        <v>46198</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>139.78</v>
+        <v>300</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I32" s="10"/>
       <c r="J32" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
@@ -21438,23 +21456,27 @@
         <v>1024</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>1014</v>
+        <v>808</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>46170</v>
+        <v>46198</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>485.13</v>
+        <v>504.19</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I33" s="10"/>
       <c r="J33" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
@@ -21470,23 +21492,27 @@
         <v>1026</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>808</v>
+        <v>1027</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>1068.45</v>
+        <v>19.78</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K34" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L34" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
@@ -21496,29 +21522,33 @@
         <v>15</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>316.46</v>
+        <v>143.08</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L35" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
@@ -21528,29 +21558,33 @@
         <v>15</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>1030</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>1031</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>1029</v>
-      </c>
       <c r="F36" s="10" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>309.58</v>
+        <v>143.08</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K36" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L36" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
@@ -21560,29 +21594,33 @@
         <v>15</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>808</v>
+        <v>1030</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>438.8</v>
+        <v>300.98</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I37" s="10"/>
       <c r="J37" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K37" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L37" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
@@ -21592,29 +21630,33 @@
         <v>15</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>1036</v>
+        <v>1030</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>350.4</v>
+        <v>300</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K38" s="11"/>
-      <c r="L38" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K38" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L38" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
@@ -21630,23 +21672,27 @@
         <v>1038</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>1039</v>
+        <v>1027</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>46198</v>
+        <v>46207</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>149.16</v>
+        <v>1154.15</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K39" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L39" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
@@ -21656,29 +21702,33 @@
         <v>15</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>1040</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>1041</v>
       </c>
-      <c r="E40" s="5" t="s">
-        <v>1029</v>
-      </c>
       <c r="F40" s="10" t="n">
-        <v>46198</v>
+        <v>46207</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>309.58</v>
+        <v>92.1</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K40" s="11"/>
-      <c r="L40" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K40" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L40" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
@@ -21694,23 +21744,27 @@
         <v>1043</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>808</v>
+        <v>995</v>
       </c>
       <c r="F41" s="10" t="n">
-        <v>46198</v>
+        <v>46231</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>837.52</v>
+        <v>487.57</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I41" s="10"/>
       <c r="J41" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K41" s="11"/>
-      <c r="L41" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K41" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L41" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
@@ -21729,20 +21783,24 @@
         <v>808</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>46198</v>
+        <v>46231</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>610.85</v>
+        <v>673.53</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K42" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L42" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
@@ -21758,23 +21816,27 @@
         <v>1047</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>1048</v>
+        <v>817</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>46198</v>
+        <v>46254</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>1617.71</v>
+        <v>576.13</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K43" s="11"/>
-      <c r="L43" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K43" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L43" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
@@ -21784,29 +21846,33 @@
         <v>15</v>
       </c>
       <c r="C44" s="5" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D44" s="5" t="s">
         <v>1049</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>1050</v>
-      </c>
       <c r="E44" s="5" t="s">
-        <v>1029</v>
+        <v>817</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>46198</v>
+        <v>46261</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>300</v>
+        <v>741.48</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K44" s="11"/>
-      <c r="L44" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K44" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L44" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
@@ -21816,29 +21882,33 @@
         <v>15</v>
       </c>
       <c r="C45" s="5" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D45" s="5" t="s">
         <v>1051</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="E45" s="5" t="s">
         <v>1052</v>
       </c>
-      <c r="E45" s="5" t="s">
-        <v>1029</v>
-      </c>
       <c r="F45" s="10" t="n">
-        <v>46198</v>
+        <v>46273</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>527.8</v>
+        <v>2518.94</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K45" s="11"/>
-      <c r="L45" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K45" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L45" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
@@ -21854,23 +21924,27 @@
         <v>1054</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>1029</v>
+        <v>1055</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>46198</v>
+        <v>46284</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>494.11</v>
+        <v>841.73</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K46" s="11"/>
-      <c r="L46" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K46" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L46" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
@@ -21880,29 +21954,33 @@
         <v>15</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>1029</v>
+        <v>834</v>
       </c>
       <c r="F47" s="10" t="n">
-        <v>46198</v>
+        <v>46284</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>300</v>
+        <v>146.86</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K47" s="11"/>
-      <c r="L47" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K47" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L47" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
@@ -21912,29 +21990,33 @@
         <v>15</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>808</v>
+        <v>834</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>46198</v>
+        <v>46284</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>504.19</v>
+        <v>146.86</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K48" s="11"/>
-      <c r="L48" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K48" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L48" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
@@ -21944,512 +22026,36 @@
         <v>15</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>1061</v>
+        <v>1055</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>46205</v>
+        <v>46284</v>
       </c>
       <c r="G49" s="6" t="n">
-        <v>19.78</v>
+        <v>711.31</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K49" s="11"/>
-      <c r="L49" s="11"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>1062</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>1063</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>1064</v>
-      </c>
-      <c r="F50" s="10" t="n">
-        <v>46205</v>
-      </c>
-      <c r="G50" s="6" t="n">
-        <v>143.08</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I50" s="10"/>
-      <c r="J50" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K50" s="11"/>
-      <c r="L50" s="11"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>1065</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>1066</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>1064</v>
-      </c>
-      <c r="F51" s="10" t="n">
-        <v>46205</v>
-      </c>
-      <c r="G51" s="6" t="n">
-        <v>143.08</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I51" s="10"/>
-      <c r="J51" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K51" s="11"/>
-      <c r="L51" s="11"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>1067</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>1068</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>1064</v>
-      </c>
-      <c r="F52" s="10" t="n">
-        <v>46205</v>
-      </c>
-      <c r="G52" s="6" t="n">
-        <v>300.98</v>
-      </c>
-      <c r="H52" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I52" s="10"/>
-      <c r="J52" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K52" s="11"/>
-      <c r="L52" s="11"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>1069</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>1070</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>1064</v>
-      </c>
-      <c r="F53" s="10" t="n">
-        <v>46205</v>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>300</v>
-      </c>
-      <c r="H53" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I53" s="10"/>
-      <c r="J53" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K53" s="11"/>
-      <c r="L53" s="11"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>1071</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>1072</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>1061</v>
-      </c>
-      <c r="F54" s="10" t="n">
-        <v>46207</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>1154.15</v>
-      </c>
-      <c r="H54" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I54" s="10"/>
-      <c r="J54" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K54" s="11"/>
-      <c r="L54" s="11"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>1073</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>1074</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>1075</v>
-      </c>
-      <c r="F55" s="10" t="n">
-        <v>46207</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>92.1</v>
-      </c>
-      <c r="H55" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I55" s="10"/>
-      <c r="J55" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K55" s="11"/>
-      <c r="L55" s="11"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>1077</v>
-      </c>
-      <c r="E56" s="5" t="s">
-        <v>1029</v>
-      </c>
-      <c r="F56" s="10" t="n">
-        <v>46231</v>
-      </c>
-      <c r="G56" s="6" t="n">
-        <v>487.57</v>
-      </c>
-      <c r="H56" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I56" s="10"/>
-      <c r="J56" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K56" s="11"/>
-      <c r="L56" s="11"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>1078</v>
-      </c>
-      <c r="D57" s="5" t="s">
-        <v>1079</v>
-      </c>
-      <c r="E57" s="5" t="s">
-        <v>808</v>
-      </c>
-      <c r="F57" s="10" t="n">
-        <v>46231</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>673.53</v>
-      </c>
-      <c r="H57" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I57" s="10"/>
-      <c r="J57" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K57" s="11"/>
-      <c r="L57" s="11"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>1080</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>1081</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>817</v>
-      </c>
-      <c r="F58" s="10" t="n">
-        <v>46254</v>
-      </c>
-      <c r="G58" s="6" t="n">
-        <v>576.13</v>
-      </c>
-      <c r="H58" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I58" s="10"/>
-      <c r="J58" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K58" s="11"/>
-      <c r="L58" s="11"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>1082</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>1083</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>817</v>
-      </c>
-      <c r="F59" s="10" t="n">
-        <v>46261</v>
-      </c>
-      <c r="G59" s="6" t="n">
-        <v>741.48</v>
-      </c>
-      <c r="H59" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I59" s="10"/>
-      <c r="J59" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K59" s="11"/>
-      <c r="L59" s="11"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>1084</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>1085</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>1086</v>
-      </c>
-      <c r="F60" s="10" t="n">
-        <v>46273</v>
-      </c>
-      <c r="G60" s="6" t="n">
-        <v>2518.94</v>
-      </c>
-      <c r="H60" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I60" s="10"/>
-      <c r="J60" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K60" s="11"/>
-      <c r="L60" s="11"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>1087</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>1088</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>1089</v>
-      </c>
-      <c r="F61" s="10" t="n">
-        <v>46284</v>
-      </c>
-      <c r="G61" s="6" t="n">
-        <v>841.73</v>
-      </c>
-      <c r="H61" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I61" s="10"/>
-      <c r="J61" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K61" s="11"/>
-      <c r="L61" s="11"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>1090</v>
-      </c>
-      <c r="D62" s="5" t="s">
-        <v>1091</v>
-      </c>
-      <c r="E62" s="5" t="s">
-        <v>834</v>
-      </c>
-      <c r="F62" s="10" t="n">
-        <v>46284</v>
-      </c>
-      <c r="G62" s="6" t="n">
-        <v>146.86</v>
-      </c>
-      <c r="H62" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I62" s="10"/>
-      <c r="J62" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K62" s="11"/>
-      <c r="L62" s="11"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>1092</v>
-      </c>
-      <c r="D63" s="5" t="s">
-        <v>1093</v>
-      </c>
-      <c r="E63" s="5" t="s">
-        <v>834</v>
-      </c>
-      <c r="F63" s="10" t="n">
-        <v>46284</v>
-      </c>
-      <c r="G63" s="6" t="n">
-        <v>146.86</v>
-      </c>
-      <c r="H63" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I63" s="10"/>
-      <c r="J63" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K63" s="11"/>
-      <c r="L63" s="11"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>1094</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>1095</v>
-      </c>
-      <c r="E64" s="5" t="s">
-        <v>1089</v>
-      </c>
-      <c r="F64" s="10" t="n">
-        <v>46284</v>
-      </c>
-      <c r="G64" s="6" t="n">
-        <v>711.31</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="I64" s="10"/>
-      <c r="J64" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="K64" s="11"/>
-      <c r="L64" s="11"/>
+        <v>964</v>
+      </c>
+      <c r="K49" s="11" t="s">
+        <v>965</v>
+      </c>
+      <c r="L49" s="11" t="s">
+        <v>966</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L64"/>
+  <autoFilter ref="A3:L49"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>